<commit_message>
Agent instructed change in graphs and tables
</commit_message>
<xml_diff>
--- a/results/ads_intensive_aggregate/estimates/ads_intensive_aggregate_b1_estimates.xlsx
+++ b/results/ads_intensive_aggregate/estimates/ads_intensive_aggregate_b1_estimates.xlsx
@@ -379,18 +379,18 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>total_shares</t>
+          <t>total_reactions</t>
         </is>
       </c>
       <c r="B2">
-        <v>-0.008560361297302956</v>
+        <v>-0.01591542146435543</v>
       </c>
       <c r="C2">
-        <v>0.02170692640002374</v>
+        <v>0.02036292150660714</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Total Shares</t>
+          <t>log(Total reactions)</t>
         </is>
       </c>
     </row>
@@ -408,25 +408,25 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Total Comments</t>
+          <t>log(Total comments)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>total_reactions</t>
+          <t>total_shares</t>
         </is>
       </c>
       <c r="B4">
-        <v>-0.01591542146435543</v>
+        <v>-0.008560361297302956</v>
       </c>
       <c r="C4">
-        <v>0.02036292150660714</v>
+        <v>0.02170692640002374</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Total Reactions</t>
+          <t>log(Total shares)</t>
         </is>
       </c>
     </row>
@@ -444,7 +444,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Verifiable Posts + Shares</t>
+          <t>log(Verifiable posts + shares)</t>
         </is>
       </c>
     </row>
@@ -462,7 +462,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Non Verifiable Posts + Shares</t>
+          <t>log(Non-verifiable posts + shares)</t>
         </is>
       </c>
     </row>
@@ -480,7 +480,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>True Posts + Shares</t>
+          <t>log(True posts + shares)</t>
         </is>
       </c>
     </row>
@@ -498,7 +498,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Fake Posts + Shares</t>
+          <t>log(Fake posts + shares)</t>
         </is>
       </c>
     </row>
@@ -516,7 +516,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Number of Posts + Shares (English)</t>
+          <t>log(Number of posts + shares, English)</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>COVID Posts + Shares</t>
+          <t>log(COVID posts + shares)</t>
         </is>
       </c>
     </row>
@@ -552,7 +552,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Positive COVID Posts + Shares</t>
+          <t>log(Positive COVID posts + shares)</t>
         </is>
       </c>
     </row>
@@ -570,7 +570,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Neutral COVID Posts + Shares</t>
+          <t>log(Neutral COVID posts + shares)</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Negative COVID Posts + Shares</t>
+          <t>log(Negative COVID posts + shares)</t>
         </is>
       </c>
     </row>
@@ -606,7 +606,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Vaccine Posts + Shares</t>
+          <t>log(Vaccine posts + shares)</t>
         </is>
       </c>
     </row>
@@ -624,7 +624,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Positive Vaccine Posts + Shares</t>
+          <t>log(Positive vaccine posts + shares)</t>
         </is>
       </c>
     </row>
@@ -642,7 +642,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Neutral Vaccine Posts + Shares</t>
+          <t>log(Neutral vaccine posts + shares)</t>
         </is>
       </c>
     </row>
@@ -660,7 +660,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Negative Vaccine Posts + Shares</t>
+          <t>log(Negative vaccine posts + shares)</t>
         </is>
       </c>
     </row>

</xml_diff>